<commit_message>
move facility dialogue into endos-junction, delete facility sheet
The facility.* lines (Endo joining, shelters, iron warnings, first
night) belong to the junction experience, not a separate "facility"
scene. Renamed to junction.* and appended to the endos-junction sheet.

The "facility" sheet name is reserved for the later attempted-return
lockout/chase arc from the GDD.

5 sheets remain: aster-sim, peris-sim, elevator, tag-day, endos-junction.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -8,7 +8,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="elevator" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tag-day" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="endos-junction" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -3931,7 +3930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4913,267 +4912,244 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>facility.exit_narration</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>junction.exit_narration</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>The facility door seals behind you. The corridor stretches ahead.</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Leaving the facility</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>facility.endo_appears</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>junction.endo_appears</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>Someone is waiting at the exit. Quiet. Watchful. He falls into step beside you.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Endo joins — no words</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>facility.endo.shelters</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>junction.endo.shelters</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>He points ahead. Then at a marker on the wall — a shelter symbol.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Endo gestures toward shelter — marker appears</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>facility.endo.iron_warn</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>junction.endo.iron_warn</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>He stops. Holds out an arm. Shakes his head slowly.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Endo blocks the iron path — marker on safe route</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>facility.endo.dusk</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>junction.endo.dusk</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>He taps the wall. Points at the dimming light. Walks faster.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Endo notices dusk — urgency without words</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>facility.endo.shelter</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>junction.endo.shelter</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>He stops at a door. Opens it. Steps aside.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Endo at the shelter entrance</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>facility.night_narration</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>junction.night_narration</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>Night. The barrier is thinner here. You can hear things moving outside.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>First night</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>facility.endo.rest</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>junction.endo.rest</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>He settles against the wall. Watches the door.</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Endo takes watch — same posture as junction</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>facility.dawn</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>junction.dawn</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Day 2. Dawn.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Morning — waits for click</t>
         </is>

</xml_diff>

<commit_message>
tag day: NK banter in dialogue box, interleaved with poem
NK chat lines now go through the dialogue box (not Label3D visuals
that weren't showing up). Single interleaved _dialogue_chain with
poem and NK lines alternating. Both driven by the same scheduler
clock via the chain mechanism.

NK speakers added to CSV: NK-01 (odd lines), NK-02 (even lines).
23-line chain: 13 poem + 10 NK chat interleaved per GDD ordering.

Dialogue box: removed scheduler reference (display-only model).
Queue depth warning at >3 entries indicates upstream timing issue.
Typewriter and hold timer use delta — upstream scheduler pushes
lines, box receives/displays/queues.

Tests: NK lines verified in dialogue log (got 10), interleaving
with poem confirmed, minimum line count raised to 33.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -3039,6 +3039,11 @@
           <t>tag_day.nk_chat.01</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3089,6 +3094,11 @@
           <t>tag_day.nk_chat.02</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3160,6 +3170,11 @@
           <t>tag_day.nk_chat.03</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3210,6 +3225,11 @@
           <t>tag_day.nk_chat.04</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3260,6 +3280,11 @@
           <t>tag_day.nk_chat.05</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3331,6 +3356,11 @@
           <t>tag_day.nk_chat.06</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3386,6 +3416,11 @@
           <t>tag_day.nk_chat.07</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3436,6 +3471,11 @@
           <t>tag_day.nk_chat.08</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3486,6 +3526,11 @@
           <t>tag_day.nk_chat.09</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>normal</t>
@@ -3533,6 +3578,11 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NK-02</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">

</xml_diff>

<commit_message>
dialogue: channels, stacks, residential rings, lockout scenes
4 new sheets in act1.xlsx (64 new dialogue lines):

Channels (20 lines): Perivascular Channels, shelters 2-3. Endo teaches
fluid reading (flowing = safe, stagnant = danger). Peris discovers flora
tending. Corpse starch introduction. Endo's gestural teaching style.

Stacks (14 lines): Processing Stacks, shelters 4-5. Aster finds raw
terminal data ("cleaned and normalized"). Information trail begins.
Myke's old workspace as retroactive environmental storytelling.

Residential Rings (15 lines): Shelters 6-7. Functioning civilization.
Peris tries to reconnect with a client through physical presence
instead of the feed. Endo departs at the furthest point from his wall.

Lockout (15 lines): The attempted return. System rejects their tags.
Aster tries to hack, triggers Naturalizers. Chase back into the
corridors. The exile is permanent.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -8,6 +8,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="elevator" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tag-day" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="endos-junction" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stacks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="residential-rings" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lockout" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -5208,4 +5212,1996 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>channels.narration.enter</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>The corridor opens. Water runs along the floor in shallow channels. The air is different here — cleaner where the water flows, stale where it pools.</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>First view of the Perivascular Channels</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>channels.aster.fluid</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fluid dynamics are still active in this section. Flow rate correlates with atmospheric quality. Where it moves, the readings are clean.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aster reads the data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>channels.peris.sound</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Listen. You can hear it. The moving water sounds different from the still water.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Peris reads by ear</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>channels.endo.stop</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>He stops at the edge of a stagnant pool. Shakes his head. Points to the flowing channel beside it.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Endo: stagnant = danger</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>channels.aster.stagnant</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Iron concentration spikes near the stagnant sections. The standing water is concentrating the deposits.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Aster confirms</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>channels.peris.thick</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>The air is heavier here. Like breathing through cloth.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Peris feels biofilm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>channels.narration.flora</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Something is growing where the water seeps into the wall. Faint. Not quite alive, not quite dead.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>First wild flora</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>channels.peris.touch</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>It responds to me. I just... touched it, and it brightened.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Peris discovers tending</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>channels.aster.glow</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bioluminescence increased by 40% on contact. Whatever you did, the growth is producing more light now.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Aster measures it</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>channels.peris.always</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>I didn't do anything. Plants just... respond to me. They always have.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>She doesn't know why</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>channels.narration.branch</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>The channels branch. One path flows steadily forward. Another leads into silence.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Route choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>channels.endo.point</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>He points toward the flowing channel. Then at the silent branch, and draws a finger across his throat.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>That way is death</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>channels.narration.body</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>A figure in the drainage channel. Still. The water flows around them. They stopped moving a long time ago.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>First lootable corpse</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>channels.endo.kneel</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>He kneels beside the body. A brief pause. Then his hands move — practiced, efficient. He stands with something in his palm.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Endo demonstrates nutrient absorption</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>channels.peris.what</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>What did he just...?</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Peris processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>channels.aster.nutrients</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Organic nutrient absorption. The biological matter still has caloric value. It is what it is.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Clinical framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>channels.peris.people</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>These were people.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Humane framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>channels.aster.hungry</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>They were. And we're hungry.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pragmatism</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>channels.narration.shelter</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A sealed alcove beside the main flow. The door responds to proximity. Inside: dry, warm, defensible.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Shelter 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>channels.endo.door</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>He opens the door. Steps aside. The same gesture as the junction.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Endo at shelter</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>stacks.narration.enter</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>The drainage channels give way to something industrial. Server racks in rows. Cooling systems humming. The sound of computation.</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Entering the Processing Stacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>stacks.aster.home</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>I know this infrastructure. These are the processing cores. Every data point I've ever analyzed was processed here.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aster recognizes the hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>stacks.peris.cold</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>It's cold in here. And loud. How does anyone work in this?</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Peris in a machine environment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>stacks.aster.terminal</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>There. A maintenance terminal. No friendly interface — just raw logs.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Raw data access</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>stacks.aster.cleaned</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>"The data has been cleaned and normalized to correct for anomalies." The same words. From my desk in the simulation.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Information trail begins</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>stacks.aster.here</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>It happened here. On these servers. Through these conduits. The system that gave me the drink machine is the same one that cleaned my reports.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Connecting the dots</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>stacks.peris.ok</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Are you OK?</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>stacks.aster.not_sure</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>I'm not sure what I expected to find. But it wasn't this.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Processing the betrayal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>stacks.narration.elegant</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>One section is noticeably better than its surroundings. The cable routing is elegant, almost artistic. Someone who cared about this hardware shaped these rows.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Myke retroactive storytelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>stacks.narration.closet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A small workspace between two racks. A half-finished schematic, crossed out and restarted in the margins. Someone was designing something better and kept stopping.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Myke was here</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stacks.aster.archive</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Older data here. The system keeps its own history in layers. I can read backwards through it.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Archive access</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>stacks.aster.when</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The normalization started on a specific date. Someone built the protocol. Someone authorized it. The terminal doesn't say who, but it shows when.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>The trail has a beginning</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>stacks.peris.meaning</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>What does that mean for us?</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>stacks.aster.means</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>It means the data isn't broken. Someone is making it wrong. On purpose.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Not failure — policy</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rings.narration.enter</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>The corridors change. Clean. Lit. Warm. People walk past on their own routines. Simulation bays glow through windows.</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Entering the Residential Rings</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>rings.aster.signal</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>System signals everywhere. Processing stations, transit routing, the full network. This is civilization.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aster reads the infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rings.peris.remember</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>I know this place. My clients lived here. The inner ones.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Peris recognizes territory</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>rings.peris.hello</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Hello? It... it's me. Peris. From the feed.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Tries to connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>rings.narration.client</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>The client looks confused. Recognizes the voice but not the face. They hurry away.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>The feed was a wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rings.peris.wall</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>The feed was supposed to connect us. It was a wall the whole time.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Peris realizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>rings.narration.empty</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Some apartments are empty. The system lists the occupants as "reassigned." Their belongings are still on the shelves.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Disappearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>rings.aster.tags</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Our tags are still flagged here. We can see all of this, but we can't participate.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ghosts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>rings.endo.discomfort</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>He's checking behind them more often. His movements are less fluid. He keeps touching the walls.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Endo far from his wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>rings.endo.stops</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>He stops. Looks back. Looks forward. Looks at them. Then turns around.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Endo chooses the wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>rings.peris.endo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Endo?</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>rings.narration.leaving</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>He doesn't explain. He's already walking back. His section of the wall needs him.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Endothelial cells don't travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>rings.peris.understands</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>I understand. Some people can only function in their own space.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Social worker reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>rings.aster.just_us</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>So it's just us now.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>rings.peris.visiting</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>It's been just us since the elevator. Endo was visiting.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Reframe: Endo was the guest</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>lockout.narration.clean</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>The corridors get cleaner. The clicking fades. The air smells filtered. Infrastructure lights improve.</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Approaching the boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>lockout.aster.signals</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>System signals are strong here. Processing stations, transit routing. We're close.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Proximity to civilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lockout.aster.panel</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Access panel. Standard interface. Let me just...</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Aster tries to interface</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>lockout.system.rejected</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NON-COMPLIANT: WELLNESS PROTOCOL DEVIATION. ACCESS REVOKED.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Rejection</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lockout.aster.again</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No. Let me try again.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Denial</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>lockout.system.rejected2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ACCESS REVOKED. REPORT TO NEAREST PROCESSING STATION.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Same result</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>lockout.aster.hack</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>I can hack it. I hacked the elevator. I can hack this.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Brute force attempt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>lockout.system.blocked</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>UNAUTHORIZED ACCESS ATTEMPT LOGGED. RESPONSE UNIT DISPATCHED.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Triggers enforcers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>lockout.narration.footsteps</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Coordinated footsteps. The scan-sweep sound. The calm efficiency of units following protocol.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Naturalizers converging</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lockout.peris.run</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>We need to go. Now.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lockout.narration.chase</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>They run. The Naturalizers don't. They walk with purpose. The gentle hands from Tag Day are reaching for them.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>The chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>lockout.narration.boundary</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The Naturalizers stop at the boundary where the system's infrastructure ends. They stand. They scan. They wait.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>The system does not extend here</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lockout.aster.not_in</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>It's not letting me back in.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>The real lockout</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lockout.peris.back_to</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>...Back in to what?</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Not rhetorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lockout.narration.forward</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>The Naturalizers watch from the boundary. The clicking of Chelators resumes behind them. There is no going back.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Exile is permanent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: merge poem stanzas so corridor walk completes before lockdown
Previous: 23 lines (13 poem + 10 NK) at 4s hold = 92s. The corridor
walk finished before the poem, and post-walk events stomped the chain.
The poem never reached the BANG fragment.

Now: 16 lines (6 merged poem stanzas + 10 NK) at 4s hold = 64s. Each
poem stanza is a single multi-line dialogue entry containing the full
couplet + refrain. Fits within the ~115s corridor walk.

Test: added "BANG fragment reached" assertion to verify the poem chain
completes and fragments fire. This would have caught the original bug.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -2897,12 +2897,13 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>tag_day.checkpoint_id</t>
-        </is>
-      </c>
+          <t>tag_day.poem.01</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -2912,522 +2913,589 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>CHECKPOINT 7-B  //  IMMUNITY VERIFICATION</t>
+          <t>Between the idea
+And the reality
+Between the motion
+And the act</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Data overlay as Aster arrives at checkpoint</t>
+          <t>First stanza — the gap between intention and action</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>tag_day.nk_chat.01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Looks like I win the bet. Not weird. He's just babbling like most of them did yesterday.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NK-01 claims victory</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>tag_day.poem.02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Falls the Shadow
+For Thine is the Kingdom</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Refrain — the Shadow falls between</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Well, it's weirdly structured, unlike all that gibberish we heard.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NK-02 pushing back</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tag_day.poem.03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Between the conception
+And the creation
+Between the emotion
+And the response</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Second stanza — the gap between feeling and acting</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>You'll call anything weird, like that case of complete silence.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NK-01 dismissing</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Silence IS weird. Yet you didn't get that hint last time you tried courtship, did you?</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NK-02 pivots to personal jab</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tag_day.poem.04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Falls the Shadow
+Life is very long</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Refrain — life stretches</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>We had three cases of silence in the last week. It's completely normal.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NK-01 deflecting with statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>...says the guy who spent his date completely silent before getting completely ghosted.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NK-02 lands the kill shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tag_day.poem.05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Between the desire
+And the spasm
+Between the potency
+And the existence
+Between the essence
+And the descent</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Third stanza — the full descent, longest breath</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>I'm working on my approach.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NK-01 retreating to vague self-improvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>You've been 'working on your approach' since orientation. How's that going?</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NK-02 won't let him have it</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tag_day.poem.06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Falls the Shadow
+For Thine is the Kingdom</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Final refrain before collapse</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>There's still time.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NK-01 down to bare assertion</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Is there? You're what, twenty-three? Twenty-four?</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NK-02 names the number — casual and terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tag_day.checkpoint_id</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CHECKPOINT 7-B  //  IMMUNITY VERIFICATION</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Data overlay as Aster arrives at checkpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>tag_day.murmur.01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Here we go round the prickly pear
 Prickly pear prickly pear</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Citizen murmuring in queue — nursery rhyme draws attention</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>tag_day.murmur.02</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Here we go round the prickly pear
 At five o'clock in the morning.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Citizen continues in queue before scan</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>tag_day.scan_failed</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>STATION 7-B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>SCAN FAILED  //  DISPATCHING RESPONSE UNIT</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Citizen's device scan fails</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>tag_day.poem.01</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Between the idea
-And the reality</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Shadow stanzas begin — corridor walk</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.01</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>NK-01</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Looks like I win the bet. Not weird. He's just babbling like most of them did yesterday.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>NK-01 claims victory — Label3D at ~4s</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>tag_day.poem.02</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Between the motion
-And the act</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.02</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NK-02</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Well, it's weirdly structured, unlike all that gibberish we heard.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>NK-02 pushing back — Label3D at ~8s</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>tag_day.poem.03</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Falls the Shadow</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>tag_day.poem.04</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>For Thine is the Kingdom</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.03</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>NK-01</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>You'll call anything weird, like that case of complete silence.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>NK-01 dismissing — Label3D at ~13s</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>tag_day.poem.05</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Between the conception
-And the creation</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.04</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>NK-02</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Silence IS weird. Yet you didn't get that hint last time you tried courtship, did you?</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>NK-02 pivots to personal jab — Label3D at ~18s</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>tag_day.poem.06</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Between the emotion
-And the response</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.05</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>NK-01</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>We had three cases of silence in the last week. It's completely normal.</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>NK-01 deflecting with statistics — Label3D at ~23s</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>tag_day.poem.07</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Falls the Shadow</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>tag_day.poem.08</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Life is very long</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.06</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>NK-02</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>...says the guy who spent his date completely silent before getting completely ghosted.</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>NK-02 lands the kill shot — Label3D at ~28s</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>tag_day.poem.09</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>poem</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Between the desire
-And the spasm</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Voice steady as they walk deeper</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tag_day.nk_chat.07</t>
+          <t>tag_day.scan_failed</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NK-01</t>
+          <t>STATION 7-B</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3437,24 +3505,25 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>I'm working on my approach.</t>
+          <t>SCAN FAILED  //  DISPATCHING RESPONSE UNIT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>NK-01 retreating to vague self-improvement — Label3D at ~33s</t>
+          <t>Citizen's device scan fails</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>tag_day.poem.10</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3464,25 +3533,25 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Between the potency
-And the existence</t>
+          <t>For Thine is</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Syntax collapsing — fragments of prayer stuttering</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>tag_day.nk_chat.08</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>NK-02</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.02</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3492,24 +3561,21 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>You've been 'working on your approach' since orientation. How's that going?</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>NK-02 won't let him have it — Label3D at ~38s</t>
-        </is>
-      </c>
+          <t>Life is</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>tag_day.poem.11</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3519,25 +3585,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Between the essence
-And the descent</t>
-        </is>
-      </c>
+          <t>For Thine is the</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tag_day.nk_chat.09</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>NK-01</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3547,24 +3609,21 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>There's still time.</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>NK-01 down to bare assertion — Label3D at ~43s</t>
-        </is>
-      </c>
+          <t>This is the way the world ends</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tag_day.poem.12</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3574,24 +3633,21 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Falls the Shadow</t>
-        </is>
-      </c>
+          <t>This is the way the world ends</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>tag_day.nk_chat.10</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>NK-02</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.06</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3601,24 +3657,21 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Is there? You're what, twenty-three? Twenty-four?</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>NK-02 names the number — casual and terminal — Label3D at ~48s</t>
-        </is>
-      </c>
+          <t>This is the way the world ends</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tag_day.poem.13</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3628,19 +3681,25 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>For Thine is the Kingdom</t>
+          <t>Not with a BANG...</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>The final line breaks mid-word</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>tag_day.fragment.01</t>
-        </is>
-      </c>
+          <t>tag_day.fragment.08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>whisper</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3650,24 +3709,25 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>For Thine is</t>
+          <t>...but a whimper.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Syntax collapsing — fragments of prayer stuttering</t>
+          <t>Muffled behind the closed door</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>tag_day.fragment.02</t>
-        </is>
-      </c>
+          <t>tag_day.lockdown</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3677,19 +3737,29 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Life is</t>
+          <t>MEDICAL BAY PROTOCOL  //  ENFORCEMENT ENABLED  //  PLEASE REMAIN IN POSITION</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Lockdown alarm after neutralization</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>tag_day.fragment.03</t>
+          <t>tag_day.groan</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BYSTANDER</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3699,19 +3769,29 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>For Thine is the</t>
+          <t>Come on... I need to get back to work.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Bystander reacting to the lockdown delay</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>tag_day.fragment.04</t>
+          <t>tag_day.report_blocked</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ASTER</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3721,19 +3801,29 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>This is the way the world ends</t>
+          <t>Ugh, can't even make an incident report.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Aster frustrated — device locked during protocol enforcement</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>tag_day.fragment.05</t>
+          <t>tag_day.scan_passed</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>STATION 7-B</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3743,19 +3833,25 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>This is the way the world ends</t>
+          <t>TAG VERIFICATION: PASSED  //  CLEARANCE NOMINAL</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Aster scans clean</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>tag_day.fragment.06</t>
-        </is>
-      </c>
+          <t>tag_day.clearance</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3765,214 +3861,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>This is the way the world ends</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>tag_day.fragment.07</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>fragment</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Not with a BANG...</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>The final line breaks mid-word</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>tag_day.fragment.08</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>whisper</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>...but a whimper.</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Muffled behind the closed door</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>tag_day.lockdown</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>MEDICAL BAY PROTOCOL  //  ENFORCEMENT ENABLED  //  PLEASE REMAIN IN POSITION</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Lockdown alarm after neutralization</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>tag_day.groan</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>BYSTANDER</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Come on... I need to get back to work.</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Bystander reacting to the lockdown delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>tag_day.report_blocked</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>ASTER</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Ugh, can't even make an incident report.</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Aster frustrated — device locked during protocol enforcement</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>tag_day.scan_passed</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>STATION 7-B</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>TAG VERIFICATION: PASSED  //  CLEARANCE NOMINAL</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Aster scans clean</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>tag_day.clearance</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
           <t>Blue light. Clean reading.</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Blue clearance — auto-advances into transition</t>
         </is>
       </c>
     </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5229,7 +5133,6 @@
           <t>channels.narration.enter</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5321,7 +5224,6 @@
           <t>channels.endo.stop</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5413,7 +5315,6 @@
           <t>channels.narration.flora</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5537,7 +5438,6 @@
           <t>channels.narration.branch</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5565,7 +5465,6 @@
           <t>channels.endo.point</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5593,7 +5492,6 @@
           <t>channels.narration.body</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5621,7 +5519,6 @@
           <t>channels.endo.kneel</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5777,7 +5674,6 @@
           <t>channels.narration.shelter</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5805,7 +5701,6 @@
           <t>channels.endo.door</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>normal</t>
@@ -5847,7 +5742,6 @@
           <t>stacks.narration.enter</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6055,7 +5949,6 @@
           <t>Are you OK?</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6095,7 +5988,6 @@
           <t>stacks.narration.elegant</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6123,7 +6015,6 @@
           <t>stacks.narration.closet</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6235,7 +6126,6 @@
           <t>What does that mean for us?</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6289,7 +6179,6 @@
           <t>rings.narration.enter</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6413,7 +6302,6 @@
           <t>rings.narration.client</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6473,7 +6361,6 @@
           <t>rings.narration.empty</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6533,7 +6420,6 @@
           <t>rings.endo.discomfort</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6561,7 +6447,6 @@
           <t>rings.endo.stops</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6609,7 +6494,6 @@
           <t>Endo?</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6617,7 +6501,6 @@
           <t>rings.narration.leaving</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>normal</t>
@@ -6697,7 +6580,6 @@
           <t>So it's just us now.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6751,7 +6633,6 @@
           <t>lockout.narration.clean</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
           <t>normal</t>
@@ -7003,7 +6884,6 @@
           <t>lockout.narration.footsteps</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>normal</t>
@@ -7051,7 +6931,6 @@
           <t>We need to go. Now.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7059,7 +6938,6 @@
           <t>lockout.narration.chase</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>normal</t>
@@ -7087,7 +6965,6 @@
           <t>lockout.narration.boundary</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>normal</t>
@@ -7179,7 +7056,6 @@
           <t>lockout.narration.forward</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>normal</t>

</xml_diff>

<commit_message>
tag day: citizen small talk before scan, Lot Clot game detail
Citizen tries small talk: "It's this time again, huh?" Aster shuts
them down: "Shh, that's against protocol." The citizen looks at him,
then turns back to the scanner. Their scan fails. The last normal
thing the citizen says before the poem begins is casual, human, and
Aster rejects it. The first hint of the simulation training out
connection.

Junction game updated to match GDD: "Lot Clot" — a sliding block
puzzle about clearing blockages from a jammed space, scratched into
the base plate in Endo's notation. Foreshadows the Mother Ferrolure
junction puzzle. Peris sees "how smooth the edges are from use."
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -2891,27 +2891,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>tag_day.citizen.talk</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CITIZEN</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>It's this time again, huh?</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Citizen tries small talk — the last normal thing they say</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>tag_day.aster.shush</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aster</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Shh, that's against protocol.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aster shuts them down — productivity over connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>tag_day.citizen.scan</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>The citizen looks at him for a moment. Then they turn back to the scanner.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>The citizen presents their tag. The scan fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>tag_day.poem.01</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Between the idea
 And the reality
@@ -2919,123 +3010,121 @@
 And the act</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>First stanza — the gap between intention and action</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>NK-01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Looks like I win the bet. Not weird. He's just babbling like most of them did yesterday.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>NK-01 claims victory</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>tag_day.poem.02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Falls the Shadow
 For Thine is the Kingdom</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Refrain — the Shadow falls between</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.02</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>NK-02</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Well, it's weirdly structured, unlike all that gibberish we heard.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>NK-02 pushing back</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>tag_day.poem.03</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Between the conception
 And the creation
@@ -3043,187 +3132,185 @@
 And the response</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Second stanza — the gap between feeling and acting</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.03</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>NK-01</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>You'll call anything weird, like that case of complete silence.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>NK-01 dismissing</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.04</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>NK-02</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Silence IS weird. Yet you didn't get that hint last time you tried courtship, did you?</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>NK-02 pivots to personal jab</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>tag_day.poem.04</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Falls the Shadow
 Life is very long</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Refrain — life stretches</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.05</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>NK-01</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>We had three cases of silence in the last week. It's completely normal.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>NK-01 deflecting with statistics</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.06</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>NK-02</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>...says the guy who spent his date completely silent before getting completely ghosted.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>NK-02 lands the kill shot</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>tag_day.poem.05</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Between the desire
 And the spasm
@@ -3233,349 +3320,265 @@
 And the descent</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Third stanza — the full descent, longest breath</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.07</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>NK-01</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>I'm working on my approach.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>NK-01 retreating to vague self-improvement</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>tag_day.nk_chat.08</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>NK-02</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>You've been 'working on your approach' since orientation. How's that going?</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>NK-02 won't let him have it</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>tag_day.poem.06</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Falls the Shadow
 For Thine is the Kingdom</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Final refrain before collapse</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.09</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>NK-01</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>There's still time.</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>NK-01 down to bare assertion</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>tag_day.nk_chat.10</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>NK-02</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Is there? You're what, twenty-three? Twenty-four?</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>NK-02 names the number — casual and terminal</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>tag_day.checkpoint_id</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>CHECKPOINT 7-B  //  IMMUNITY VERIFICATION</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Data overlay as Aster arrives at checkpoint</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>tag_day.nk_chat.09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NK-01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>There's still time.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NK-01 down to bare assertion</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tag_day.nk_chat.10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NK-02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Is there? You're what, twenty-three? Twenty-four?</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NK-02 names the number — casual and terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tag_day.checkpoint_id</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CHECKPOINT 7-B  //  IMMUNITY VERIFICATION</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Data overlay as Aster arrives at checkpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>tag_day.murmur.01</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Here we go round the prickly pear
 Prickly pear prickly pear</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Citizen murmuring in queue — nursery rhyme draws attention</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>tag_day.murmur.02</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>poem</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Here we go round the prickly pear
 At five o'clock in the morning.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Citizen continues in queue before scan</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>tag_day.scan_failed</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>STATION 7-B</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SCAN FAILED  //  DISPATCHING RESPONSE UNIT</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Citizen's device scan fails</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>tag_day.fragment.01</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>fragment</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>For Thine is</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Syntax collapsing — fragments of prayer stuttering</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>tag_day.fragment.02</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>fragment</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Life is</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>tag_day.fragment.03</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
+          <t>tag_day.scan_failed</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>STATION 7-B</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3585,18 +3588,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>For Thine is the</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>SCAN FAILED  //  DISPATCHING RESPONSE UNIT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Citizen's device scan fails</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tag_day.fragment.04</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>tag_day.fragment.01</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>fragment</t>
@@ -3609,18 +3615,21 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>This is the way the world ends</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>For Thine is</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Syntax collapsing — fragments of prayer stuttering</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tag_day.fragment.05</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
+          <t>tag_day.fragment.02</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>fragment</t>
@@ -3633,18 +3642,16 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>This is the way the world ends</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>Life is</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>tag_day.fragment.06</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>tag_day.fragment.03</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>fragment</t>
@@ -3657,18 +3664,16 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>This is the way the world ends</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>For Thine is the</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tag_day.fragment.07</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>tag_day.fragment.04</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>fragment</t>
@@ -3681,25 +3686,19 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Not with a BANG...</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>The final line breaks mid-word</t>
+          <t>This is the way the world ends</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>tag_day.fragment.08</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>tag_day.fragment.05</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>whisper</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3709,25 +3708,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>...but a whimper.</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Muffled behind the closed door</t>
+          <t>This is the way the world ends</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>tag_day.lockdown</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>tag_day.fragment.06</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3737,29 +3730,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>MEDICAL BAY PROTOCOL  //  ENFORCEMENT ENABLED  //  PLEASE REMAIN IN POSITION</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Lockdown alarm after neutralization</t>
+          <t>This is the way the world ends</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>tag_day.groan</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>BYSTANDER</t>
+          <t>tag_day.fragment.07</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3769,29 +3752,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Come on... I need to get back to work.</t>
+          <t>Not with a BANG...</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bystander reacting to the lockdown delay</t>
+          <t>The final line breaks mid-word</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>tag_day.report_blocked</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>ASTER</t>
+          <t>tag_day.fragment.08</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>whisper</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3801,24 +3779,19 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ugh, can't even make an incident report.</t>
+          <t>...but a whimper.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Aster frustrated — device locked during protocol enforcement</t>
+          <t>Muffled behind the closed door</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>tag_day.scan_passed</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>STATION 7-B</t>
+          <t>tag_day.lockdown</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3833,50 +3806,138 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>TAG VERIFICATION: PASSED  //  CLEARANCE NOMINAL</t>
+          <t>MEDICAL BAY PROTOCOL  //  ENFORCEMENT ENABLED  //  PLEASE REMAIN IN POSITION</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aster scans clean</t>
+          <t>Lockdown alarm after neutralization</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>tag_day.groan</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BYSTANDER</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Come on... I need to get back to work.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Bystander reacting to the lockdown delay</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tag_day.report_blocked</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ASTER</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Ugh, can't even make an incident report.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Aster frustrated — device locked during protocol enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tag_day.scan_passed</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>STATION 7-B</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TAG VERIFICATION: PASSED  //  CLEARANCE NOMINAL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Aster scans clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>tag_day.clearance</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>Blue light. Clean reading.</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Blue clearance — auto-advances into transition</t>
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4330,7 +4391,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aster at the puzzle game — can't fathom leisure_x000d_</t>
+          <t>Aster can't fathom leisure — "Lot Clot" scratched into the base plate</t>
         </is>
       </c>
     </row>
@@ -4357,12 +4418,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oh, it's a little puzzle. Someone made this by hand. It's been used a lot, look how smooth the edges are.</t>
+          <t>Oh, it's a little puzzle. Someone made this by hand. Look how smooth the edges are from use.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Peris at the puzzle game — she sees the care and the loneliness_x000d_</t>
+          <t>Peris sees the care and the years of play — sliding block puzzle about clearing blockages</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
remove elevator lockout dialogue, defer to act1 attempted return
Removed NON-COMPLIANT notification, dismiss, "not back", and "forward"
dialogue from the elevator. Characters don't discover they're locked
out until the act1 Residential Rings scene when they try to re-enter.

Doors open now leads straight to multiselect tutorial.
Removed duplicate has_override test variable.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -1612,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2344,17 +2344,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>elevator.system.noncompliant</t>
+          <t>elevator.peris.not_supposed</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SYSTEM</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2364,19 +2364,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TAG STATUS: NON-COMPLIANT  //  WELLNESS PROTOCOL DEVIATION</t>
+          <t>I don't think we're supposed to be here.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Notification Aster dismisses — not a lockout yet_x000d_</t>
+          <t>Entering the maintenance corridor_x000d_</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>elevator.aster.dismiss</t>
+          <t>elevator.aster.no_service</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2396,24 +2396,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Administrative error. I'll sort it out when we get back.</t>
+          <t>Nobody is. This section hasn't been serviced in... the maintenance logs just stop.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Aster doesn't understand what non-compliant means yet_x000d_</t>
+          <t>Aster reads corridor data_x000d_</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>elevator.peris.not_back</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Peris</t>
+          <t>elevator.bridge.narration</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2428,24 +2423,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>I don't really have anything to go back to, anyways...</t>
+          <t>An elevated walkway spanning a larger space. Incomplete railing. Exposed framework. The air is open — it smells like rust.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>_x000d_</t>
+          <t>Bridge description_x000d_</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>elevator.aster.forward</t>
+          <t>elevator.peris.bodies</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2460,24 +2455,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Forward then.</t>
+          <t>Those people down there...</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>_x000d_</t>
+          <t>Peris sees bodies below the bridge_x000d_</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>elevator.peris.not_supposed</t>
+          <t>elevator.aster.logs</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2492,19 +2487,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>I don't think we're supposed to be here.</t>
+          <t>All casualties are supposed to be logged. I'll check the records when we find a working terminal. Come on.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Entering the maintenance corridor_x000d_</t>
+          <t>Aster files it as data and keeps moving_x000d_</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>elevator.aster.no_service</t>
+          <t>elevator.aster.ahead</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2514,29 +2509,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Nobody is. This section hasn't been serviced in... the maintenance logs just stop.</t>
+          <t>There's something ahead. Lights.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Aster reads corridor data_x000d_</t>
+          <t>Waits for click — bridge collapse follows_x000d_</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>elevator.bridge.narration</t>
+          <t>elevator.peris.floor</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2551,19 +2551,19 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>An elevated walkway spanning a larger space. Incomplete railing. Exposed framework. The air is open — it smells like rust.</t>
+          <t>The floor—!</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bridge description_x000d_</t>
+          <t>Bridge gives way_x000d_</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>elevator.peris.bodies</t>
+          <t>elevator.peris.hurt</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2583,19 +2583,19 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Those people down there...</t>
+          <t>Are you hurt?</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Peris sees bodies below the bridge_x000d_</t>
+          <t>After the fall_x000d_</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>elevator.aster.logs</t>
+          <t>elevator.aster.sublevel</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2615,19 +2615,19 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>All casualties are supposed to be logged. I'll check the records when we find a working terminal. Come on.</t>
+          <t>Sub-level. We fell through.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aster files it as data and keeps moving_x000d_</t>
+          <t>Aster reads the environment_x000d_</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>elevator.aster.ahead</t>
+          <t>elevator.aster.climb</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2642,24 +2642,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>There's something ahead. Lights.</t>
+          <t>They might have called me a beast, but I'm not this type of animal...</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Waits for click — bridge collapse follows_x000d_</t>
+          <t>Looking up at the collapsed bridge — no way back up_x000d_</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>elevator.peris.floor</t>
+          <t>elevator.peris.climb</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2679,29 +2679,29 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>The floor—!</t>
+          <t>We've got the combined strength of two children. It wouldn't be physically possible to climb this...</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Bridge gives way_x000d_</t>
+          <t>_x000d_</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>elevator.peris.hurt</t>
+          <t>elevator.aster.another_way</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2711,19 +2711,19 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Are you hurt?</t>
+          <t>There's something over there. Another way forward.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>After the fall_x000d_</t>
+          <t>Finds the alternative path (TBD)_x000d_</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>elevator.aster.sublevel</t>
+          <t>elevator.aster.two_paths</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2743,138 +2743,10 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sub-level. We fell through.</t>
+          <t>Two corridors. One's clear but corroded. The other's shorter, but something's in there.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
-        <is>
-          <t>Aster reads the environment_x000d_</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>elevator.aster.climb</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Aster</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>They might have called me a beast, but I'm not this type of animal...</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Looking up at the collapsed bridge — no way back up_x000d_</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>elevator.peris.climb</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Peris</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>We've got the combined strength of two children. It wouldn't be physically possible to climb this...</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>elevator.aster.another_way</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Aster</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>There's something over there. Another way forward.</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Finds the alternative path (TBD)_x000d_</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>elevator.aster.two_paths</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Aster</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Two corridors. One's clear but corroded. The other's shorter, but something's in there.</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
         <is>
           <t>Aster reads the fork — safe route has iron hazards on floor; dangerous route has hostiles</t>
         </is>
@@ -2964,7 +2836,6 @@
           <t>tag_day.citizen.scan</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>normal</t>

</xml_diff>

<commit_message>
use real newlines in xlsx, drop pipe separator for xlsx loader
xlsx cells support native newlines — the pipe hack was only
needed for Godot CSV parsing. Replaced all remaining pipes
in act1.xlsx with actual newlines. Removed the pipe-to-newline
replacement from the xlsx loading path (kept in CSV fallback).
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -3557,7 +3557,9 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>This is the way the world ends|This is the way the world ends|This is the way the world ends</t>
+          <t>This is the way the world ends
+This is the way the world ends
+This is the way the world ends</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
clean xlsx: remove em dashes, _x000d_ artifacts, tighten contexts
Replaced all em dashes in dialogue text: interruptions use ...
(trailing off), system readouts use // (established separator).
Removed 94 _x000d_ carriage return artifacts from context column.
Cleared empty/redundant context entries. No em dashes remain
in the workbook. 477/477 pass.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Aster frustrated at desk — model isn't working_x000d_</t>
+          <t>Aster frustrated at desk - model isn't working</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Institutional stonewalling — he's trying to do better work_x000d_</t>
+          <t>Institutional stonewalling - he's trying to do better work</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ron checks his device as he walks up_x000d_</t>
+          <t>Ron checks his device as he walks up</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Ron glances at device — read the name off it_x000d_</t>
+          <t>Ron glances at device, reads the name off it</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Ron genuinely curious — sets up Aster showing the terminal_x000d_</t>
+          <t>Ron asks Aster about his work</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Tutorial beat: player moves Aster to terminal_x000d_</t>
+          <t>Tutorial: player moves Aster to terminal</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Visible on terminal — set dressing now; most important sentence later_x000d_</t>
+          <t>Message on terminal (will be replaced by GUI and other message about crediting support team)</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Ron tying initiative to perks — institutional carrot_x000d_</t>
+          <t>Ron praises Aster, brings up drink machine</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Label that appears over the drink machine during tutorial_x000d_</t>
+          <t>Label that appears over the drink machine during tutorial</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Soft redirect if player wanders away from drink machine_x000d_</t>
+          <t>Soft redirect if player wanders away from drink machine</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>The motto — directive disguised as camaraderie_x000d_</t>
+          <t>"Move fast and break things" but it's broken lol</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TAG VERIFICATION — CHECKPOINT 7-B — REPORT WITHIN 15 MINUTES</t>
+          <t>TAG VERIFICATION // CHECKPOINT 7-B // REPORT WITHIN 15 MINUTES</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Device notification_x000d_</t>
+          <t>Device notification</t>
         </is>
       </c>
     </row>
@@ -843,7 +843,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Ron reacts to the device notification_x000d_</t>
+          <t>Ron reacts to the device notification</t>
         </is>
       </c>
     </row>
@@ -865,12 +865,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Time for Tag Day. Routine.</t>
+          <t>Man, they should really automate these checks sometime...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aster's flat reaction — waits for player click</t>
+          <t>Aster reacts</t>
         </is>
       </c>
     </row>
@@ -914,11 +914,6 @@
           <t>text</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>context_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -943,7 +938,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Peris at her desk waiting for client_x000d_</t>
+          <t>Peris at her desk waiting for client</t>
         </is>
       </c>
     </row>
@@ -970,12 +965,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sorry I'm late. Sorry. I was — there was someone following me.</t>
+          <t>Sorry I'm late. Sorry. I was... there was someone following me.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Monos arrives flustered through the portal_x000d_</t>
+          <t>Monos arrives flustered through the portal</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1002,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Trailing off — the fear he didn't lose them_x000d_</t>
+          <t>Trailing off - the fear he didn't lose them</t>
         </is>
       </c>
     </row>
@@ -1037,11 +1032,6 @@
           <t>Anyway. I'm here now. Let's start.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1071,7 +1061,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Session opener — casual warmth_x000d_</t>
+          <t>Session opener - casual warmth</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1093,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Monos tired — not elaborating_x000d_</t>
+          <t>Monos tired - not elaborating</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1125,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Monos can't relax_x000d_</t>
+          <t>Monos can't relax</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1157,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Peris reassuring_x000d_</t>
+          <t>Peris reassuring</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1189,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Trying to compose himself_x000d_</t>
+          <t>Trying to compose himself</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1221,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Ready to begin the session_x000d_</t>
+          <t>Ready to begin the session</t>
         </is>
       </c>
     </row>
@@ -1258,12 +1248,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>—!</t>
+          <t>...!</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Attack through the portal — Monos is hurt_x000d_</t>
+          <t>Attack through the portal - Monos is hurt</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1285,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mandatory compliance warning — not optional_x000d_</t>
+          <t>Mandatory compliance warning - not optional</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1317,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Peris's instinct — first ability is care_x000d_</t>
+          <t>Peris's instinct - first ability is care</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1344,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Urgency — player must run to portal_x000d_</t>
+          <t>Urgency - player must run to portal</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1371,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Soft redirect if player ignores Monos — Peris's care ethic_x000d_</t>
+          <t>Soft redirect if player ignores Monos - Peris's care ethic</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1398,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Redirect if player tries ability out of range_x000d_</t>
+          <t>Redirect if player tries ability out of range</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1425,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Player tried to run before queuing protect_x000d_</t>
+          <t>Player tried to run before queuing protect</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1452,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Player clicked somewhere other than near Monos_x000d_</t>
+          <t>Player clicked somewhere other than near Monos</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1479,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Player tried to unpause too early_x000d_</t>
+          <t>Player tried to unpause too early</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1501,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wait — I need to queue the ability first.</t>
+          <t>Wait... I need to queue the ability first.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Player tried to unpause before queuing protect_x000d_</t>
+          <t>Player tried to unpause before queuing protect</t>
         </is>
       </c>
     </row>
@@ -1546,11 +1536,6 @@
           <t>I... thank you. I don't know what that was. Thank you, Peris.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1575,12 +1560,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SESSION COMPLETE — EFFICIENCY: 62%  //  OVERTIME PENALTY LOGGED</t>
+          <t>SESSION COMPLETE // EFFICIENCY: 62% // OVERTIME PENALTY LOGGED</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Efficiency penalty_x000d_</t>
+          <t>Efficiency penalty</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1582,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Session ends — portal closes and Monos fades out</t>
+          <t>Session ends - portal closes and Monos fades out</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1628,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Peris wakes in the elevator_x000d_</t>
+          <t>Peris wakes in the elevator</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1655,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Scene description_x000d_</t>
+          <t>Scene description</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1687,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Peris approaches Aster_x000d_</t>
+          <t>Peris approaches Aster</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1719,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Aster wakes groggy — still in the simulation mentally_x000d_</t>
+          <t>Aster wakes groggy - still in the simulation mentally</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1751,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aster realizes_x000d_</t>
+          <t>Aster realizes</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1783,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aster checks device first thing_x000d_</t>
+          <t>Aster checks device first thing</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1815,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Peris confirms they're stuck_x000d_</t>
+          <t>Peris confirms they're stuck</t>
         </is>
       </c>
     </row>
@@ -1860,11 +1845,6 @@
           <t>Why are we here?</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1894,7 +1874,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aster retells it flatly — doesn't know what happened_x000d_</t>
+          <t>Aster retells it flatly - doesn't know what happened</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1906,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No mention of the bang — Aster's data view couldn't see the room_x000d_</t>
+          <t>No mention of the bang - Aster's data view couldn't see the room</t>
         </is>
       </c>
     </row>
@@ -1956,11 +1936,6 @@
           <t>Is he OK?</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1990,7 +1965,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Cites the policy like it settles the matter_x000d_</t>
+          <t>Cites the policy like it settles the matter</t>
         </is>
       </c>
     </row>
@@ -2022,7 +1997,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Pivots — policy is also what happened to her_x000d_</t>
+          <t>Pivots - policy is also what happened to her</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2029,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Peris disturbed by how soothing it was meant to be_x000d_</t>
+          <t>Peris disturbed by how soothing it was meant to be</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2061,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Oblivious flex — interrupted by system restoration_x000d_</t>
+          <t>Oblivious flex - interrupted by system restoration</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2093,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>System restores devices and wakes escorts simultaneously_x000d_</t>
+          <t>System restores devices and wakes escorts simultaneously</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2125,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aster's data overlay reveals the panel_x000d_</t>
+          <t>Aster's data overlay reveals the panel</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2157,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Escort units activate as part of the same restoration_x000d_</t>
+          <t>Escort units activate as part of the same restoration</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2189,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Aster panicking but finding a solution_x000d_</t>
+          <t>Aster panicking but finding a solution</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2221,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Post-EMP urgency_x000d_</t>
+          <t>Post-EMP urgency</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2253,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Aster begins hacking the panel_x000d_</t>
+          <t>Aster begins hacking the panel</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2285,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Hack succeeds_x000d_</t>
+          <t>Hack succeeds</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2312,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Doors open_x000d_</t>
+          <t>Doors open</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2344,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Entering the maintenance corridor_x000d_</t>
+          <t>Entering the maintenance corridor</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2376,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Aster reads corridor data_x000d_</t>
+          <t>Aster reads corridor data</t>
         </is>
       </c>
     </row>
@@ -2423,12 +2398,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>An elevated walkway spanning a larger space. Incomplete railing. Exposed framework. The air is open — it smells like rust.</t>
+          <t>An elevated walkway spanning a larger space. Incomplete railing. Exposed framework. The air is open -- it smells like rust.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Bridge description_x000d_</t>
+          <t>Bridge description</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2435,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Peris sees bodies below the bridge_x000d_</t>
+          <t>Peris sees bodies below the bridge</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2467,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Aster files it as data and keeps moving_x000d_</t>
+          <t>Aster files it as data and keeps moving</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2499,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Waits for click — bridge collapse follows_x000d_</t>
+          <t>Waits for click - bridge collapse follows</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2526,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>The floor—!</t>
+          <t>The floor...!</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bridge gives way_x000d_</t>
+          <t>Bridge gives way</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2563,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>After the fall_x000d_</t>
+          <t>After the fall</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2595,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aster reads the environment_x000d_</t>
+          <t>Aster reads the environment</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2627,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Looking up at the collapsed bridge — no way back up_x000d_</t>
+          <t>Looking up at the collapsed bridge - no way back up</t>
         </is>
       </c>
     </row>
@@ -2682,11 +2657,6 @@
           <t>We've got the combined strength of two children. It wouldn't be physically possible to climb this...</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2716,7 +2686,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Finds the alternative path (TBD)_x000d_</t>
+          <t>Finds the alternative path (TBD)</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2718,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Aster reads the fork — safe route has iron hazards on floor; dangerous route has hostiles</t>
+          <t>Aster reads the fork - safe route has iron hazards on floor; dangerous route has hostiles</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2764,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Citizen tries small talk — the last normal thing they say</t>
+          <t>Citizen tries small talk - the last normal thing they say</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2796,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Aster shuts them down — productivity over connection</t>
+          <t>Aster shuts them down - productivity over connection</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2853,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>First stanza — the gap between intention and action</t>
+          <t>First stanza - the gap between intention and action</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2913,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Refrain — the Shadow falls between</t>
+          <t>Refrain - the Shadow falls between</t>
         </is>
       </c>
     </row>
@@ -3005,7 +2975,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Second stanza — the gap between feeling and acting</t>
+          <t>Second stanza - the gap between feeling and acting</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3067,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Refrain — life stretches</t>
+          <t>Refrain - life stretches</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3163,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Third stanza — the full descent, longest breath</t>
+          <t>Third stanza - the full descent, longest breath</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3319,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>NK-02 names the number — casual and terminal</t>
+          <t>NK-02 names the number - casual and terminal</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3374,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Citizen murmuring in queue — nursery rhyme draws attention</t>
+          <t>Citizen murmuring in queue - nursery rhyme draws attention</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3461,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Syntax collapsing — fragments of prayer stuttering</t>
+          <t>Syntax collapsing - fragments of prayer stuttering</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3674,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aster frustrated — device locked during protocol enforcement</t>
+          <t>Aster frustrated - device locked during protocol enforcement</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3733,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Blue clearance — auto-advances into transition</t>
+          <t>Blue clearance - auto-advances into transition</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3774,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Scripted dusk — first nightfall approaching_x000d_</t>
+          <t>Scripted dusk - first nightfall approaching</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3806,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Aster examines the workbench_x000d_</t>
+          <t>Aster examines the workbench</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3838,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Peris examines the workbench_x000d_</t>
+          <t>Peris examines the workbench</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3870,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Aster reads the monitoring station_x000d_</t>
+          <t>Aster reads the monitoring station</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3902,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Peris reads the monitoring station_x000d_</t>
+          <t>Peris reads the monitoring station</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3934,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aster at the food cache — compliance over survival_x000d_</t>
+          <t>Aster at the food cache - compliance over survival</t>
         </is>
       </c>
     </row>
@@ -3996,7 +3966,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Peris at the food cache — empathy over survival_x000d_</t>
+          <t>Peris at the food cache - empathy over survival</t>
         </is>
       </c>
     </row>
@@ -4028,7 +3998,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Aster at the lookout spot_x000d_</t>
+          <t>Aster at the lookout spot</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4030,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Peris at the lookout spot_x000d_</t>
+          <t>Peris at the lookout spot</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4062,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Aster at the heater — data without emotional inference_x000d_</t>
+          <t>Aster at the heater - data without emotional inference</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4094,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Peris at the heater — she reads the care_x000d_</t>
+          <t>Peris at the heater - she reads the care</t>
         </is>
       </c>
     </row>
@@ -4156,7 +4126,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Aster at the wall markings — unrecognized system_x000d_</t>
+          <t>Aster at the wall markings - unrecognized system</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4158,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Peris at the wall markings — she reads the person_x000d_</t>
+          <t>Peris at the wall markings - she reads the person</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4190,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aster can't fathom leisure — "Lot Clot" scratched into the base plate</t>
+          <t>Aster can't fathom leisure - "Lot Clot" scratched into the base plate</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4222,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Peris sees the care and the years of play — sliding block puzzle about clearing blockages</t>
+          <t>Peris sees the care and the years of play - sliding block puzzle about clearing blockages</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4249,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Endo gestures them inside — marker appears on shelter_x000d_</t>
+          <t>Endo gestures them inside - marker appears on shelter</t>
         </is>
       </c>
     </row>
@@ -4309,11 +4279,6 @@
           <t>Who...?</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4343,7 +4308,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Aster scans Endo_x000d_</t>
+          <t>Aster scans Endo</t>
         </is>
       </c>
     </row>
@@ -4370,7 +4335,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Endo offers drink — marker on container_x000d_</t>
+          <t>Endo offers drink - marker on container</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4367,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Accepts the drink_x000d_</t>
+          <t>Accepts the drink</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4394,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Endo takes watch — no marker needed_x000d_</t>
+          <t>Endo takes watch - no marker needed</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4421,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Pairs of eyes outside — the player sees them too_x000d_</t>
+          <t>Pairs of eyes outside - the player sees them too</t>
         </is>
       </c>
     </row>
@@ -4483,7 +4448,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>The eyes recede with the light_x000d_</t>
+          <t>The eyes recede with the light</t>
         </is>
       </c>
     </row>
@@ -4510,7 +4475,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Evidence of the night visitors_x000d_</t>
+          <t>Evidence of the night visitors</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4507,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Aster tries his device — locked out of the simulation_x000d_</t>
+          <t>Aster tries his device - locked out of the simulation</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4539,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Not rhetorical — what exactly does he want to go back to_x000d_</t>
+          <t>Not rhetorical - what exactly does he want to go back to</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4566,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Endo gestures: he's coming with_x000d_</t>
+          <t>Endo gestures: he's coming with</t>
         </is>
       </c>
     </row>
@@ -4631,11 +4596,6 @@
           <t>I think he's coming with us.</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4663,11 +4623,6 @@
           <t>I don't see why not.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>_x000d_</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4697,7 +4652,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aster reads the gauntlet_x000d_</t>
+          <t>Aster reads the gauntlet</t>
         </is>
       </c>
     </row>
@@ -4724,12 +4679,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>There's something on the wall. Iron lure — ferrolure. If I activate it, they might go for that instead.</t>
+          <t>There's something on the wall. Iron lure -- ferrolure. If I activate it, they might go for that instead.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Peris recognizes the device_x000d_</t>
+          <t>Peris recognizes the device</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4765,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Endo joins — no words</t>
+          <t>Endo joins - no words</t>
         </is>
       </c>
     </row>
@@ -4832,12 +4787,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>He points ahead. Then at a marker on the wall — a shelter symbol.</t>
+          <t>He points ahead. Then at a marker on the wall -- a shelter symbol.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Endo gestures toward shelter — marker appears</t>
+          <t>Endo gestures toward shelter - marker appears</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4819,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Endo blocks the iron path — marker on safe route</t>
+          <t>Endo blocks the iron path - marker on safe route</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4846,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Endo notices dusk — urgency without words</t>
+          <t>Endo notices dusk - urgency without words</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4927,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Endo takes watch — same posture as junction</t>
+          <t>Endo takes watch - same posture as junction</t>
         </is>
       </c>
     </row>
@@ -4999,7 +4954,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Morning — waits for click</t>
+          <t>Morning - waits for click</t>
         </is>
       </c>
     </row>
@@ -5035,7 +4990,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>The corridor opens. Water runs along the floor in shallow channels. The air is different here — cleaner where the water flows, stale where it pools.</t>
+          <t>The corridor opens. Water runs along the floor in shallow channels. The air is different here -- cleaner where the water flows, stale where it pools.</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5421,7 +5376,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>He kneels beside the body. A brief pause. Then his hands move — practiced, efficient. He stands with something in his palm.</t>
+          <t>He kneels beside the body. A brief pause. Then his hands move -- practiced, efficient. He stands with something in his palm.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -5740,7 +5695,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>There. A maintenance terminal. No friendly interface — just raw logs.</t>
+          <t>There. A maintenance terminal. No friendly interface -- just raw logs.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -6045,7 +6000,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Not failure — policy</t>
+          <t>Not failure - policy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
remove back_in/back_to_what dialogue from morning sequence
Removed junction.aster.back_in and junction.peris.back_to_what
from the xlsx and the morning dialogue chain. Morning now goes
straight from trail evidence to Endo standing up and the party
leaving. 477/477 pass.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -3748,7 +3748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4482,12 +4482,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>junction.aster.back_in</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Aster</t>
+          <t>junction.endo.stands</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4502,19 +4497,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>It's not letting me back in.</t>
+          <t>He stands. Looks at the corridor ahead, then at them. Steps toward the door.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Aster tries his device - locked out of the simulation</t>
+          <t>Endo gestures: he's coming with</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>junction.peris.back_to_what</t>
+          <t>junction.peris.coming</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4534,19 +4529,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>...Back in to what?</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Not rhetorical - what exactly does he want to go back to</t>
+          <t>I think he's coming with us.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>junction.endo.stands</t>
+          <t>junction.aster.ok</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4561,29 +4556,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>He stands. Looks at the corridor ahead, then at them. Steps toward the door.</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Endo gestures: he's coming with</t>
+          <t>I don't see why not.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>junction.peris.coming</t>
+          <t>junction.aster.blocked</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -4593,19 +4583,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>I think he's coming with us.</t>
+          <t>Dense cluster ahead. Five, maybe six. Too many to push through.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Aster reads the gauntlet</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>junction.aster.ok</t>
+          <t>junction.peris.ferrolure</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4620,19 +4615,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>I don't see why not.</t>
+          <t>There's something on the wall. Iron lure -- ferrolure. If I activate it, they might go for that instead.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Peris recognizes the device</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>junction.aster.blocked</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Aster</t>
+          <t>junction.ferrolure.active</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4647,24 +4642,19 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Dense cluster ahead. Five, maybe six. Too many to push through.</t>
+          <t>FERROLURE ACTIVE  //  SIDEROPHORE LURE  //  18s REMAINING</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aster reads the gauntlet</t>
+          <t>System readout</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>junction.peris.ferrolure</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Peris</t>
+          <t>junction.exit_narration</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4679,24 +4669,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>There's something on the wall. Iron lure -- ferrolure. If I activate it, they might go for that instead.</t>
+          <t>The facility door seals behind you. The corridor stretches ahead.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Peris recognizes the device</t>
+          <t>Leaving the facility</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>junction.ferrolure.active</t>
+          <t>junction.endo_appears</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4706,19 +4696,19 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FERROLURE ACTIVE  //  SIDEROPHORE LURE  //  18s REMAINING</t>
+          <t>Someone is waiting at the exit. Quiet. Watchful. He falls into step beside you.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>System readout</t>
+          <t>Endo joins - no words</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>junction.exit_narration</t>
+          <t>junction.endo.shelters</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -4733,19 +4723,19 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>The facility door seals behind you. The corridor stretches ahead.</t>
+          <t>He points ahead. Then at a marker on the wall -- a shelter symbol.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Leaving the facility</t>
+          <t>Endo gestures toward shelter - marker appears</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>junction.endo_appears</t>
+          <t>junction.endo.iron_warn</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4760,19 +4750,19 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Someone is waiting at the exit. Quiet. Watchful. He falls into step beside you.</t>
+          <t>He stops. Holds out an arm. Shakes his head slowly.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Endo joins - no words</t>
+          <t>Endo blocks the iron path - marker on safe route</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>junction.endo.shelters</t>
+          <t>junction.endo.dusk</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4787,19 +4777,19 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>He points ahead. Then at a marker on the wall -- a shelter symbol.</t>
+          <t>He taps the wall. Points at the dimming light. Walks faster.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Endo gestures toward shelter - marker appears</t>
+          <t>Endo notices dusk - urgency without words</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>junction.endo.iron_warn</t>
+          <t>junction.endo.shelter</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4814,19 +4804,19 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>He stops. Holds out an arm. Shakes his head slowly.</t>
+          <t>He stops at a door. Opens it. Steps aside.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Endo blocks the iron path - marker on safe route</t>
+          <t>Endo at the shelter entrance</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>junction.endo.dusk</t>
+          <t>junction.night_narration</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4841,19 +4831,19 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>He taps the wall. Points at the dimming light. Walks faster.</t>
+          <t>Night. The barrier is thinner here. You can hear things moving outside.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Endo notices dusk - urgency without words</t>
+          <t>First night</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>junction.endo.shelter</t>
+          <t>junction.endo.rest</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4868,91 +4858,37 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>He stops at a door. Opens it. Steps aside.</t>
+          <t>He settles against the wall. Watches the door.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Endo at the shelter entrance</t>
+          <t>Endo takes watch - same posture as junction</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>junction.night_narration</t>
+          <t>junction.dawn</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Night. The barrier is thinner here. You can hear things moving outside.</t>
+          <t>Day 2. Dawn.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
-        <is>
-          <t>First night</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>junction.endo.rest</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>He settles against the wall. Watches the door.</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Endo takes watch - same posture as junction</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>junction.dawn</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Day 2. Dawn.</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
         <is>
           <t>Morning - waits for click</t>
         </is>

</xml_diff>

<commit_message>
plant triggers Endo, chunk jumping, AnimationPlayer infrastructure
Peris tending the dormant plant at Endo's junction triggers dusk
and Endo's arrival (was an arbitrary 8s timer). Plant blooms with
bioluminescence on interaction, ambient light fades to dusk, Endo
appears from the shadows 2s later.

Scene chunking moved to base class (TutorialSequence._load_chunk,
_unload_chunk, _build_chunk). Subclasses override _build_chunk
with a match dispatch. Both elevator and act1 have start_chunk
export: set to "junction" or "stacks" in the inspector to skip
directly to any chunk for testing.

AnimationPlayer infrastructure in base class: _create_animation,
_play_animation, speed_scale synced with scheduler in _process.
Complements existing tweens for reusable named sequences.

New dialogue: junction.peris.tend_plant ("Something's still alive
in here. Just barely."). 478/478 pass.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -3849,7 +3849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3887,7 +3887,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>junction.dusk</t>
+          <t>junction.peris.tend_plant</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3902,29 +3907,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The light is changing. Dimming.</t>
+          <t>Something's still alive in here. Just barely.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Scripted dusk - first nightfall approaching</t>
+          <t>Peris tends the dormant plant, triggering dusk</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>junction.workbench.aster</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Aster</t>
+          <t>junction.dusk</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3934,29 +3934,29 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sealant applicators. Pressure readers. Manual torque adjusters. No automated systems. Whoever lives here is maintaining this entire section by hand.</t>
+          <t>The light is changing. Dimming.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Aster examines the workbench</t>
+          <t>Scripted dusk - first nightfall approaching</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>junction.workbench.peris</t>
+          <t>junction.workbench.aster</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3966,29 +3966,29 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>These are all laid out so carefully. Every tool in its place. Someone really cares about their work.</t>
+          <t>Sealant applicators. Pressure readers. Manual torque adjusters. No automated systems. Whoever lives here is maintaining this entire section by hand.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Peris examines the workbench</t>
+          <t>Aster examines the workbench</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>junction.monitor.aster</t>
+          <t>junction.workbench.peris</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3998,29 +3998,29 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Barrier integrity readings. Trending downward. Slowly, but consistently. Whoever is logging this has been watching the wall weaken for years.</t>
+          <t>These are all laid out so carefully. Every tool in its place. Someone really cares about their work.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aster reads the monitoring station</t>
+          <t>Peris examines the workbench</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>junction.monitor.peris</t>
+          <t>junction.monitor.aster</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4030,24 +4030,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>All these little gauges. I don't know what they measure but they all look like they're... leaning the wrong way.</t>
+          <t>Barrier integrity readings. Trending downward. Slowly, but consistently. Whoever is logging this has been watching the wall weaken for years.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Peris reads the monitoring station</t>
+          <t>Aster reads the monitoring station</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>junction.food.aster</t>
+          <t>junction.monitor.peris</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4062,24 +4062,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Consuming food you do not own is a breach of protocol.</t>
+          <t>All these little gauges. I don't know what they measure but they all look like they're... leaning the wrong way.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Aster at the food cache - compliance over survival</t>
+          <t>Peris reads the monitoring station</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>junction.food.peris</t>
+          <t>junction.food.aster</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4094,29 +4094,29 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>It's not very nice to take someone else's food!</t>
+          <t>Consuming food you do not own is a breach of protocol.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Peris at the food cache - empathy over survival</t>
+          <t>Aster at the food cache and makes a Chrono Trigger reference</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>junction.lookout.aster</t>
+          <t>junction.food.peris</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4126,29 +4126,29 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Significant wear pattern on the floor here. Someone stands in this exact spot regularly. The window faces the bridge approach.</t>
+          <t>It's not very nice to take someone else's food!</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aster at the lookout spot</t>
+          <t>I'm still mad I got all guilty during the Chrono Trigger trial scene for trying to experience the game. How Heidiggerian of me lmao</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>junction.lookout.peris</t>
+          <t>junction.lookout.aster</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4158,29 +4158,29 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Someone stands here a lot. Looking out. Waiting for someone.</t>
+          <t>Significant wear pattern on the floor here. Someone stands in this exact spot regularly. The window faces the bridge approach.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Peris at the lookout spot</t>
+          <t>Aster at the lookout spot</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>junction.heater.aster</t>
+          <t>junction.lookout.peris</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4190,29 +4190,29 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>This heating element is active and positioned at the entrance. Inefficient placement for personal use. It's oriented outward.</t>
+          <t>Someone stands here a lot. Looking out. Waiting for someone.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Aster at the heater - data without emotional inference</t>
+          <t>Peris at the lookout spot</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>junction.heater.peris</t>
+          <t>junction.heater.aster</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4222,29 +4222,29 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>This is warm. It's been running for a while. Someone set it up for visitors.</t>
+          <t>This heating element is active and positioned at the entrance. Inefficient placement for personal use. It's oriented outward.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Peris at the heater - she reads the care</t>
+          <t>My electric bill is rolling in its grave</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>junction.markings.aster</t>
+          <t>junction.heater.peris</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4254,29 +4254,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>What annotation format is this? This is definitely not standard!</t>
+          <t>This is warm. It's been running for a while. Someone set it up for visitors.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Aster at the wall markings - unrecognized system</t>
+          <t>Peris at the heater - she reads the care</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>junction.markings.peris</t>
+          <t>junction.markings.aster</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4286,24 +4286,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>I'm not sure what these markings say, but the handwriting's got a lot of personality.</t>
+          <t>What annotation format is this? This is definitely not standard!</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Peris at the wall markings - she reads the person</t>
+          <t>Aster at the wall markings - unrecognized system</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>junction.game.aster</t>
+          <t>junction.markings.peris</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4318,24 +4318,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Who has time to waste on things like these?</t>
+          <t>I'm not sure what these markings say, but the handwriting's got a lot of personality.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Aster can't fathom leisure - "Lot Clot" scratched into the base plate</t>
+          <t>Peris at the wall markings - she reads the person</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>junction.game.peris</t>
+          <t>junction.game.aster</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4350,19 +4350,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oh, it's a little puzzle. Someone made this by hand. Look how smooth the edges are from use.</t>
+          <t>Who has time to waste on things like these?</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Peris sees the care and the years of play - sliding block puzzle about clearing blockages</t>
+          <t>Aster can't fathom leisure - "Lot Clot" scratched into the base plate</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>junction.endo.beckon</t>
+          <t>junction.game.peris</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4377,24 +4382,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Someone in the doorway. Beckoning.</t>
+          <t>Oh, it's a little puzzle. Someone made this by hand. Look how smooth the edges are from use.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Endo gestures them inside - marker appears on shelter</t>
+          <t>Peris sees the care and the years of play - sliding block puzzle about clearing blockages</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>junction.peris.who</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Peris</t>
+          <t>junction.endo.beckon</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4409,24 +4409,29 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Who...?</t>
+          <t>Someone in the doorway. Beckoning.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Endo gestures them inside - marker appears on shelter</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>junction.aster.endo_read</t>
+          <t>junction.peris.who</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4436,24 +4441,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Endosomal unit. Non-hostile. His tag reads compliant, but the signal's dead.</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Aster scans Endo</t>
+          <t>Who...?</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>junction.endo.drink</t>
+          <t>junction.aster.endo_read</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4463,24 +4468,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>He holds out a container. Points at it, then at them.</t>
+          <t>Endosomal unit. Non-hostile. His tag reads compliant, but the signal's dead.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Endo offers drink - marker on container</t>
+          <t>Aster scans Endo</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>junction.peris.stomach</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Peris</t>
+          <t>junction.endo.drink</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4495,19 +4495,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Can't sleep well on an empty stomach.</t>
+          <t>He holds out a container. Points at it, then at them.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Accepts the drink</t>
+          <t>Endo offers drink - marker on container</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>junction.endo.rest</t>
+          <t>junction.peris.stomach</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4522,24 +4527,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>He moves to the window. Settles against the wall, watching outward.</t>
+          <t>Can't sleep well on an empty stomach.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Endo takes watch - no marker needed</t>
+          <t>Accepts the drink</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>junction.night.eyes</t>
+          <t>junction.endo.rest</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4549,24 +4554,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Red. Through the grating. Watching.</t>
+          <t>He moves to the window. Settles against the wall, watching outward.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Pairs of eyes outside - the player sees them too</t>
+          <t>Endo takes watch - no marker needed</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>junction.dawn</t>
+          <t>junction.night.eyes</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -4576,19 +4581,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Morning. They're gone.</t>
+          <t>Red. Through the grating. Watching.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>The eyes recede with the light</t>
+          <t>Pairs of eyes outside - the player sees them too</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>junction.morning.trail</t>
+          <t>junction.dawn</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4603,19 +4608,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A faint wet trail near the shelter door, already drying. It wasn't there last night.</t>
+          <t>Morning. They're gone.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Evidence of the night visitors</t>
+          <t>The eyes recede with the light</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>junction.endo.stands</t>
+          <t>junction.morning.trail</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -4630,24 +4635,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>He stands. Looks at the corridor ahead, then at them. Steps toward the door.</t>
+          <t>A faint wet trail near the shelter door, already drying. It wasn't there last night.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Endo gestures: he's coming with</t>
+          <t>Evidence of the night visitors</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>junction.peris.coming</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Peris</t>
+          <t>junction.endo.stands</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4662,19 +4662,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>I think he's coming with us.</t>
+          <t>He stands. Looks at the corridor ahead, then at them. Steps toward the door.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Endo gestures: he's coming with</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>junction.aster.ok</t>
+          <t>junction.peris.coming</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aster</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4689,14 +4694,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>I don't see why not.</t>
+          <t>I think he's coming with us.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>junction.aster.blocked</t>
+          <t>junction.aster.ok</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4706,7 +4711,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -4716,29 +4721,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Dense cluster ahead. Five, maybe six. Too many to push through.</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Aster reads the gauntlet</t>
+          <t>I don't see why not.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>junction.peris.ferrolure</t>
+          <t>junction.aster.blocked</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>Aster</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -4748,24 +4748,29 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>There's something on the wall. Iron lure -- ferrolure. If I activate it, they might go for that instead.</t>
+          <t>Dense cluster ahead. Five, maybe six. Too many to push through.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Peris recognizes the device</t>
+          <t>Aster reads the gauntlet</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>junction.ferrolure.active</t>
+          <t>junction.peris.ferrolure</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4775,24 +4780,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FERROLURE ACTIVE  //  SIDEROPHORE LURE  //  18s REMAINING</t>
+          <t>There's something on the wall. Iron lure -- ferrolure. If I activate it, they might go for that instead.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>System readout</t>
+          <t>Peris recognizes the device</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>junction.exit_narration</t>
+          <t>junction.ferrolure.active</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4802,19 +4807,19 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>The facility door seals behind you. The corridor stretches ahead.</t>
+          <t>FERROLURE ACTIVE  //  SIDEROPHORE LURE  //  18s REMAINING</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Leaving the facility</t>
+          <t>System readout</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>junction.endo_appears</t>
+          <t>junction.exit_narration</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -4829,19 +4834,19 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Someone is waiting at the exit. Quiet. Watchful. He falls into step beside you.</t>
+          <t>The facility door seals behind you. The corridor stretches ahead.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Endo joins - no words</t>
+          <t>Leaving the facility</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>junction.endo.shelters</t>
+          <t>junction.endo_appears</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4856,19 +4861,19 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>He points ahead. Then at a marker on the wall -- a shelter symbol.</t>
+          <t>Someone is waiting at the exit. Quiet. Watchful. He falls into step beside you.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Endo gestures toward shelter - marker appears</t>
+          <t>Endo joins - no words</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>junction.endo.iron_warn</t>
+          <t>junction.endo.shelters</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4883,19 +4888,19 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>He stops. Holds out an arm. Shakes his head slowly.</t>
+          <t>He points ahead. Then at a marker on the wall -- a shelter symbol.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Endo blocks the iron path - marker on safe route</t>
+          <t>Endo gestures toward shelter - marker appears</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>junction.endo.dusk</t>
+          <t>junction.endo.iron_warn</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4910,19 +4915,19 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>He taps the wall. Points at the dimming light. Walks faster.</t>
+          <t>He stops. Holds out an arm. Shakes his head slowly.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Endo notices dusk - urgency without words</t>
+          <t>Endo blocks the iron path - marker on safe route</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>junction.endo.shelter</t>
+          <t>junction.endo.dusk</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4937,19 +4942,19 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>He stops at a door. Opens it. Steps aside.</t>
+          <t>He taps the wall. Points at the dimming light. Walks faster.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Endo at the shelter entrance</t>
+          <t>Endo notices dusk - urgency without words</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>junction.night_narration</t>
+          <t>junction.endo.shelter</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4964,19 +4969,19 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Night. The barrier is thinner here. You can hear things moving outside.</t>
+          <t>He stops at a door. Opens it. Steps aside.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>First night</t>
+          <t>Endo at the shelter entrance</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>junction.endo.rest</t>
+          <t>junction.night_narration</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4991,37 +4996,64 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>He settles against the wall. Watches the door.</t>
+          <t>Night. The barrier is thinner here. You can hear things moving outside.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Endo takes watch - same posture as junction</t>
+          <t>First night</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>junction.endo.rest</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>He settles against the wall. Watches the door.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Endo takes watch - same posture as junction</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>junction.dawn</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Day 2. Dawn.</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Morning - waits for click</t>
         </is>

</xml_diff>

<commit_message>
dialogue: user copy edits and peris_sim scene updates
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -1483,7 +1483,7 @@
         <v>false</v>
       </c>
       <c r="E18" t="str">
-        <v>My device. It's back. There's a maintenance panel behind the doors.</v>
+        <v>Looks like my perks are coming in handy. There's a maintenance panel behind the doors!</v>
       </c>
       <c r="F18" t="str">
         <v>Aster's data overlay reveals the panel</v>
@@ -1523,10 +1523,10 @@
         <v>false</v>
       </c>
       <c r="E20" t="str">
-        <v>No no no. My device. I can pulse it, fry their circuits.</v>
+        <v>Hey, want to see a perk I haven't tried yet?</v>
       </c>
       <c r="F20" t="str">
-        <v>Aster panicking but finding a solution</v>
+        <v>Aster about to use EMP</v>
       </c>
     </row>
     <row r="21">
@@ -1800,7 +1800,7 @@
         <v>They might have called me a beast, but I'm not this type of animal...</v>
       </c>
       <c r="F34" t="str">
-        <v>Looking up at the collapsed bridge - no way back up</v>
+        <v xml:space="preserve">This is totally a reference to Reanimal </v>
       </c>
     </row>
     <row r="35">
@@ -1819,6 +1819,9 @@
       <c r="E35" t="str">
         <v>We've got the combined strength of two children. It wouldn't be physically possible to climb this...</v>
       </c>
+      <c r="F35" t="str">
+        <v>I loved Reanimal but those kids were built different</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1834,10 +1837,10 @@
         <v>false</v>
       </c>
       <c r="E36" t="str">
-        <v>There's something over there. Another way forward.</v>
+        <v>Huh, looks like there's [TBD] though...</v>
       </c>
       <c r="F36" t="str">
-        <v>Finds the alternative path (TBD)</v>
+        <v>Something is found in the cracks (TBD)</v>
       </c>
     </row>
     <row r="37">
@@ -2221,7 +2224,7 @@
 For Thine is the Kingdom</v>
       </c>
       <c r="F18" t="str">
-        <v>Final refrain before collapse</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -2241,7 +2244,7 @@
         <v>There's still time.</v>
       </c>
       <c r="F19" t="str">
-        <v>NK-01 down to bare assertion</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -2261,7 +2264,7 @@
         <v>Is there? You're what, twenty-three? Twenty-four?</v>
       </c>
       <c r="F20" t="str">
-        <v>NK-02 names the number - casual and terminal</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2296,7 +2299,7 @@
 Prickly pear prickly pear</v>
       </c>
       <c r="F22" t="str">
-        <v>Citizen murmuring in queue - nursery rhyme draws attention</v>
+        <v>Time for T.S. Elliot, thanks public domain</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -2314,7 +2317,7 @@
 At five o'clock in the morning.</v>
       </c>
       <c r="F23" t="str">
-        <v>Citizen continues in queue before scan</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -2351,7 +2354,7 @@
         <v>For Thine is</v>
       </c>
       <c r="F25" t="str">
-        <v>Syntax collapsing - fragments of prayer stuttering</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -2608,7 +2611,7 @@
         <v>false</v>
       </c>
       <c r="E4" t="str">
-        <v>Sealant applicators. Pressure readers. Manual torque adjusters. No automated systems. Whoever lives here is maintaining this entire section by hand.</v>
+        <v>Sealant applicators. Pressure readers. Manual torque adjusters. Looks like someone missed the automation assisance memo...</v>
       </c>
       <c r="F4" t="str">
         <v>Aster examines the workbench</v>
@@ -2628,10 +2631,10 @@
         <v>false</v>
       </c>
       <c r="E5" t="str">
-        <v>These are all laid out so carefully. Every tool in its place. Someone really cares about their work.</v>
+        <v>I remember a client saying they keep their home neat because it reflects the values they'd want to show in the outside world. I wonder if someone's doing the same?</v>
       </c>
       <c r="F5" t="str">
-        <v>Peris examines the workbench</v>
+        <v>Peris examines workbench (Thanks Arendt for the discussion of private vs. public and the invasion of the social in The Human Condition)</v>
       </c>
     </row>
     <row r="6">
@@ -2648,7 +2651,7 @@
         <v>false</v>
       </c>
       <c r="E6" t="str">
-        <v>Barrier integrity readings. Trending downward. Slowly, but consistently. Whoever is logging this has been watching the wall weaken for years.</v>
+        <v>Why are these barrier integrity readings still going down? I thought the other team was assigned to this!</v>
       </c>
       <c r="F6" t="str">
         <v>Aster reads the monitoring station</v>
@@ -2668,7 +2671,7 @@
         <v>false</v>
       </c>
       <c r="E7" t="str">
-        <v>All these little gauges. I don't know what they measure but they all look like they're... leaning the wrong way.</v>
+        <v>I bet Aster would know how to read these! All I can read is how antsy he seems...</v>
       </c>
       <c r="F7" t="str">
         <v>Peris reads the monitoring station</v>
@@ -2688,7 +2691,7 @@
         <v>false</v>
       </c>
       <c r="E8" t="str">
-        <v>Consuming food you do not own is a breach of protocol.</v>
+        <v>Consuming food you do not own is a breach of protocol. Would look awful in a trial.</v>
       </c>
       <c r="F8" t="str">
         <v>Aster at the food cache and makes a Chrono Trigger reference</v>
@@ -2728,7 +2731,7 @@
         <v>false</v>
       </c>
       <c r="E10" t="str">
-        <v>Significant wear pattern on the floor here. Someone stands in this exact spot regularly. The window faces the bridge approach.</v>
+        <v>Ugh, look at the mess outside. At least whoever lives here seems to be competent...</v>
       </c>
       <c r="F10" t="str">
         <v>Aster at the lookout spot</v>
@@ -2748,7 +2751,7 @@
         <v>false</v>
       </c>
       <c r="E11" t="str">
-        <v>Someone stands here a lot. Looking out. Waiting for someone.</v>
+        <v>Look at the view! It's like what I've seen through client portals!</v>
       </c>
       <c r="F11" t="str">
         <v>Peris at the lookout spot</v>
@@ -2768,7 +2771,7 @@
         <v>false</v>
       </c>
       <c r="E12" t="str">
-        <v>This heating element is active and positioned at the entrance. Inefficient placement for personal use. It's oriented outward.</v>
+        <v>A heater right next to the entrance? The heat's going to leak right out!</v>
       </c>
       <c r="F12" t="str">
         <v>My electric bill is rolling in its grave</v>
@@ -2788,7 +2791,7 @@
         <v>false</v>
       </c>
       <c r="E13" t="str">
-        <v>This is warm. It's been running for a while. Someone set it up for visitors.</v>
+        <v>Looks like someone wanted to give a warm welcome!</v>
       </c>
       <c r="F13" t="str">
         <v>Peris at the heater - she reads the care</v>
@@ -2848,7 +2851,7 @@
         <v>false</v>
       </c>
       <c r="E16" t="str">
-        <v>Who has time to waste on things like these?</v>
+        <v>*Lot Clot*. Who has time to waste on things like these? Glad they invented portals and working *in simulo*...</v>
       </c>
       <c r="F16" t="str">
         <v>Aster can't fathom leisure - "Lot Clot" scratched into the base plate</v>
@@ -2868,7 +2871,7 @@
         <v>false</v>
       </c>
       <c r="E17" t="str">
-        <v>Oh, it's a little puzzle. Someone made this by hand. Look how smooth the edges are from use.</v>
+        <v>*Lot Clot*. Ooh, a traffic jam? Vehicles? How vintage!</v>
       </c>
       <c r="F17" t="str">
         <v>Peris sees the care and the years of play - sliding block puzzle about clearing blockages</v>
@@ -2885,7 +2888,7 @@
         <v>false</v>
       </c>
       <c r="E18" t="str">
-        <v>Someone in the doorway. Beckoning.</v>
+        <v>Hey, someone's here!</v>
       </c>
       <c r="F18" t="str">
         <v>Endo gestures them inside - marker appears on shelter</v>

</xml_diff>

<commit_message>
dialogue: save user edits before script modification
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -2774,7 +2774,7 @@
         <v>A heater right next to the entrance? The heat's going to leak right out!</v>
       </c>
       <c r="F12" t="str">
-        <v>My electric bill is rolling in its grave</v>
+        <v>Aster at the heater (My electric bill is rolling in its grave)</v>
       </c>
     </row>
     <row r="13">
@@ -2794,7 +2794,7 @@
         <v>Looks like someone wanted to give a warm welcome!</v>
       </c>
       <c r="F13" t="str">
-        <v>Peris at the heater - she reads the care</v>
+        <v>Peris at the heater</v>
       </c>
     </row>
     <row r="14">
@@ -2814,7 +2814,7 @@
         <v>What annotation format is this? This is definitely not standard!</v>
       </c>
       <c r="F14" t="str">
-        <v>Aster at the wall markings - unrecognized system</v>
+        <v>Aster at the wall markings</v>
       </c>
     </row>
     <row r="15">
@@ -2834,7 +2834,7 @@
         <v>I'm not sure what these markings say, but the handwriting's got a lot of personality.</v>
       </c>
       <c r="F15" t="str">
-        <v>Peris at the wall markings - she reads the person</v>
+        <v>Peris at the wall markings</v>
       </c>
     </row>
     <row r="16">
@@ -2854,7 +2854,7 @@
         <v>*Lot Clot*. Who has time to waste on things like these? Glad they invented portals and working *in simulo*...</v>
       </c>
       <c r="F16" t="str">
-        <v>Aster can't fathom leisure - "Lot Clot" scratched into the base plate</v>
+        <v>Aster Peris reacts to "Lot Clot"</v>
       </c>
     </row>
     <row r="17">
@@ -2874,7 +2874,7 @@
         <v>*Lot Clot*. Ooh, a traffic jam? Vehicles? How vintage!</v>
       </c>
       <c r="F17" t="str">
-        <v>Peris sees the care and the years of play - sliding block puzzle about clearing blockages</v>
+        <v>Peris reacts to "Lot Clot"</v>
       </c>
     </row>
     <row r="18">
@@ -3362,7 +3362,7 @@
         <v>Fluid dynamics are still active in this section. Flow rate correlates with atmospheric quality. Where it moves, the readings are clean.</v>
       </c>
       <c r="F3" t="str">
-        <v>Aster reads the data</v>
+        <v>Aster analyzes fluid</v>
       </c>
     </row>
     <row r="4">
@@ -3382,7 +3382,7 @@
         <v>Listen. You can hear it. The moving water sounds different from the still water.</v>
       </c>
       <c r="F4" t="str">
-        <v>Peris reads by ear</v>
+        <v>Peris hears the fluid</v>
       </c>
     </row>
     <row r="5">
@@ -3641,7 +3641,7 @@
         <v>false</v>
       </c>
       <c r="E18" t="str">
-        <v>These were people.</v>
+        <v>These were people...</v>
       </c>
       <c r="F18" t="str">
         <v>Humane framing</v>
@@ -3661,7 +3661,7 @@
         <v>false</v>
       </c>
       <c r="E19" t="str">
-        <v>They were. And we're hungry.</v>
+        <v>And these will be us if we don't eat! It's a downgrade for me too, you know...</v>
       </c>
       <c r="F19" t="str">
         <v>Pragmatism</v>

</xml_diff>

<commit_message>
control prompts name the LIVE binding: 'Click' becomes 'Right-click' (InputLabels)
The interactable hint still said 'Click' from the left-click era. Rather than
hard-coding the new button, prompts derive from the InputMap:

- InputLabels (scripts/ui): action_label() names an action's current binding
  (mouse buttons -> 'Right-click' etc., keys via the OS keycode string), and
  expand() substitutes '{action}' tokens in any text — so a rebind (or another
  controls overhaul) can never strand stale instructions on screen.
- The interactable's default floating hint is action_label('command') ->
  'Right-click'; explicit labels run through expand().
- The drink machine's xlsx label becomes the '{command}' token (with a context
  note for translators) instead of the literal 'click'.
- Guarded: the highlight suite asserts the default names the live binding and
  that token expansion works.

syntax, aster sim, input playthrough, interactable highlight green (544).
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -612,12 +612,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>click</t>
+          <t>{command}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Label that appears over the drink machine during tutorial</t>
+          <t>Floating control hint over the drink machine; {command} substitutes the live interact binding (right-click on desktop).</t>
         </is>
       </c>
     </row>
@@ -9109,7 +9109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
dialogue: add the watering/habit line + Peris plant-text edits
Adds peris.sim_expand.plant_7.line (the watering-tradition line: 'people used to water
their plants because it helped them have a sense of time, growth and habit maintenance')
+ plant_7.look (the watering-action narration) + plant_7.line_repeat, and refreshes the
plant_1/5/9 texts.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -10246,7 +10246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10887,12 +10887,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>This one's doing so well! I wasn't sure she'd take when I moved her from the hallway, but she's really settled in. Look at how she's leaning toward the light...</t>
+          <t>Growing plants is a dying art nowadays. It used to be such a trend when I was young, and everyone wanted the simple life of maintenance work.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Pilea peperomioides (Chinese money plant)</t>
+          <t>Register: reflective, gently nostalgic. Voice direction: Peris is speaking to herself while touching a leaf. 'A dying art' is delivered matter-of-factly. 'Such a trend when I was young' is small private nostalgia. 'Everyone wanted the simple life of maintenance work' is delivered straight; Peris was drawn to it then and still values it now. (Replaces the original Pilea 'doing so well / leaning toward the light' line; reassigned in the May 31 design session, propagated here from the transcript record.)</t>
         </is>
       </c>
     </row>
@@ -11015,12 +11015,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oh, this one's from a client! They got curious about the game after seeing it in my office. Ended up really getting into it. We did a swap last spring.</t>
+          <t>Oh, this one's from a client! They got curious about the game after seeing it in my office. Ended up really getting into it. We did a swap last spring. Sweet person. They were really into curecumin too, kept some of the old natural stuff in a hidden cabinet in their home, the kind that opens and closes three times in a row to reveal the compartment. They told me once, like it was a small secret.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Pothos (Epipremnum aureum)</t>
+          <t>Pothos (Epipremnum aureum). Register: warm, conversationally proud, then slightly nostalgic in the curecumin beat. SEED (load-bearing, do not trim): the curecumin-cabinet detail teaches the unguessable open-and-close-three-times mechanism for a permanent stat-boost reward (a Curecumin jar) found in the Teacher's home in the Act 2 Outer Homes scene. The line is the only place that mechanism is taught; a player who skips it cannot solve the cabinet on first contact. Delivered as a fond client memory, not a treasure hint. Client is the Teacher archetype but is not named here, preserving the Act 2 reveal. The curecumin half was previously dropped from this cell and is restored verbatim from simulation_tutorial_expansions.</t>
         </is>
       </c>
     </row>
@@ -11059,12 +11059,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>peris.sim_expand.plant_7.line</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Peris</t>
+          <t>peris.sim_expand.plant_7.look</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -11079,19 +11074,19 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Maybe she's just fussy because she feels far from what she's used to. If it's too wet, she gets upset. If it's too dry, then she'll cry. She needs what she needs.</t>
+          <t>Peris notices the watering can on the shelf. She picks it up, holds it a moment, and tips it gently over the soil.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Boston fern (Nephrolepis exaltata)</t>
+          <t>Approach and teaching beat. This is where the tutorial teaches item-use and the hand-inventory slot: Peris picks up the watering can (item enters the hand slot), then uses it on the plant (item-use on a target). The everyday motion of someone who waters regularly; the mechanic is taught through her habit, not through a prompt she narrates.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>peris.sim_expand.plant_8.line</t>
+          <t>peris.sim_expand.plant_7.line</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -11111,19 +11106,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oh, this one's actually named after one of my clients! Kindest person. Knew how to fix things nobody else could figure out. My whole game broke one morning, all my plants turned into pink blocks, and he came over and sorted it all out. I haven't been out to see him in a while... I should schedule a visit soon.</t>
+          <t>Did you know that people used to water their plants because it helped them have a sense of time, growth and habit maintenance? Such a beautiful tradition!</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Spider plant (Chlorophytum comosum)</t>
+          <t>Register: warm, share-trivia-with-delight, affectionate. Voice direction: Peris is sharing a small fact she finds lovely, the way she might share an anecdote with a client. 'Did you know' opens with her gentle inclusive register. 'Such a beautiful tradition!' closes with real appreciation; the exclamation is felt, not performed. The misunderstanding (that plants do not in fact die without water) lives in what the line does not say: Peris frames watering purely as ritual and habit, never as survival, and never registers that the omission is an omission. Her plants are engineered to stay green, so she has no reference for plants dying from lack of water. The misunderstanding lands on the player, not on her. Carries the engineered-green-plants reveal. (Replaces the retired fern empathy-mirror beat; per the May 31 design session this slot was reassigned from the Boston fern to the watering reflection.)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>peris.sim_expand.plant_9.line</t>
+          <t>peris.sim_expand.plant_7.line_repeat</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -11143,19 +11138,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>I remember when I was a kid, and this plant game was so popular! My clients and I still love it. Makes for a great atmosphere.</t>
+          <t>I read once that some people even kept a little log of it. What day, how much. Imagine caring for something that carefully, just to mark the time passing.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Peace lily (Spathiphyllum)</t>
+          <t>Fires on re-interaction with plant_7 (after the tradition line). Continues the watering-tradition thread and keeps the misunderstanding load-bearing: Peris still frames watering as pure ritual, never as survival. 'Just to mark the time passing' reinforces that the water does nothing the plant needs, in her understanding; her plants are engineered to stay green. Trigger: repeat interaction only, not first contact.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>peris.sim_expand.painting.line</t>
+          <t>peris.sim_expand.plant_8.line</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -11175,19 +11170,19 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>The vibes of this painting really brighten up the room! I wonder if artists ever enjoy their work as much as the people who look at it?</t>
+          <t>Oh, this one's actually named after one of my clients! Kindest person. Knew how to fix things nobody else could figure out. My whole game broke one morning, all my plants turned into pink blocks, and he came over and sorted it all out. I haven't been out to see him in a while... I should schedule a visit soon.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Empathic reach past her clients to a stranger; 'too' nearly acknowledges her own needs</t>
+          <t>Spider plant (Chlorophytum comosum)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>peris.sim_expand.wellness.line</t>
+          <t>peris.sim_expand.plant_9.line</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -11207,24 +11202,29 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>'Take a breath.' 'You deserve a moment.' You know what'd help? If I could replace these with photos of my clients...</t>
+          <t>I remember when this plant game was the thing, when I was a kid! It's old now, I know. My clients and I still love it anyway. They don't make them like they used to.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sets up the sanction-arc replacement of her feed with this exact content</t>
+          <t>Peace lily (Spathiphyllum). Register: enthusiastic, nostalgic, warmly conversational; the most energetically-voiced line in the workspace, a deliberate spike up from her low-key plant register. PAYOFF: establishes Peris's affection for the vintage plant game, which pays off when she reacts with delight to Endo's Clot Lot game at the junction ('Ooh! How vintage!'). 'My clients and I still love it' is the load-bearing phrase: the game is a shared aesthetic touchpoint across years of her clients. Pairs with plant_5, which makes that shared-touchpoint specific via one client who took up the game.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>peris.sim_expand.strike_warning.notification</t>
+          <t>peris.sim_expand.painting.line</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ui</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -11234,19 +11234,19 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WORKFORCE CONDUCT STATUS: WARNING (2/3 VIOLATIONS)</t>
+          <t>The vibes of this painting really brighten up the room! I wonder if artists ever enjoy their work as much as the people who look at it?</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Compliance document; shorter UI register without heavy separator punctuation</t>
+          <t>Empathic reach past her clients to a stranger; 'too' nearly acknowledges her own needs</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>peris.sim_expand.strike_warning.line</t>
+          <t>peris.sim_expand.wellness.line</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -11266,29 +11266,24 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>In my defense, the sessions get cut off way too quickly! Only the newer, younger therapists need that much time. I write my notes in a third of the time they give me...</t>
+          <t>'Take a breath.' 'You deserve a moment.' You know what'd help? If I could replace these with photos of my clients...</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Deflecting joke that still reveals why the warning exists without spelling out the stakes</t>
+          <t>Sets up the sanction-arc replacement of her feed with this exact content</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>peris_sim.system.sanction_notice</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
+          <t>peris.sim_expand.strike_warning.notification</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>ui</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -11298,29 +11293,29 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ROLE PRIVILEGES REVOKED. ENABLING SAFEGUARD MODE</t>
+          <t>WORKFORCE CONDUCT STATUS: WARNING (2/3 VIOLATIONS)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Peris receives her final strike after saving Monos.</t>
+          <t>Compliance document; shorter UI register without heavy separator punctuation</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>peris_sim.system.wellness_feed</t>
+          <t>peris.sim_expand.strike_warning.line</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SYSTEM</t>
+          <t>Peris</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -11330,29 +11325,29 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>3-Step Mindset Mastery: Techniques for handling stress...</t>
+          <t>In my defense, the sessions get cut off way too quickly! Only the newer, younger therapists need that much time. I write my notes in a third of the time they give me...</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>The sanction portal replaces client work with wellness prompts and satisfying content.</t>
+          <t>Deflecting joke that still reveals why the warning exists without spelling out the stakes</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>peris_sim.peris.sanction_reaction</t>
+          <t>peris_sim.system.sanction_notice</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PERIS</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -11362,24 +11357,29 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>The only steps I need are more ones around this room...</t>
+          <t>ROLE PRIVILEGES REVOKED. ENABLING SAFEGUARD MODE</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Peris reacts to sanction mode.</t>
+          <t>Peris receives her final strike after saving Monos.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>peris_sim.system.spiral_flash</t>
+          <t>peris_sim.system.wellness_feed</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>fragment</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -11389,24 +11389,24 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>For one frame, the gel loop tears open into spirals. Then the soap-cutting video resumes, seamless and soft.</t>
+          <t>3-Step Mindset Mastery: Techniques for handling stress...</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>The spiralverse leaks through the wellness footage for a single frame, the gel loop tearing into spirals before the soothing video reseals. The spiral is the capture motif (the Psyknapse trap, the spiralverse); here it surfaces inside the comfort content, a glimpse of what the wellness layer sits on top of.</t>
+          <t>The sanction portal replaces client work with wellness prompts and satisfying content.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>peris_sim.peris.retro</t>
+          <t>peris_sim.peris.sanction_reaction</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Peris</t>
+          <t>PERIS</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -11421,29 +11421,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>What even is all this? Looks like some really retro footage...</t>
+          <t>The only steps I need are more ones around this room...</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Peris's reaction to the glitch. She does not register the spiral as an intrusion at all; she takes it for part of the footage, just more dated, odd wellness video. The dark irony is that the capture motif surfaces right in front of her and reads to her as nothing, content.</t>
+          <t>Peris reacts to sanction mode.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>peris_sim.worker.okay</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>WORKER</t>
+          <t>peris_sim.system.spiral_flash</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>fragment</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -11453,42 +11448,106 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Hey, we detected abnormal vital signals. Let's get you looked at.</t>
+          <t>For one frame, the gel loop tears open into spirals. Then the soap-cutting video resumes, seamless and soft.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Adjacent worker reacts as Peris removes the sim equipment.</t>
+          <t>The spiralverse leaks through the wellness footage for a single frame, the gel loop tearing into spirals before the soothing video reseals. The spiral is the capture motif (the Psyknapse trap, the spiralverse); here it surfaces inside the comfort content, a glimpse of what the wellness layer sits on top of.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>peris_sim.peris.retro</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Peris</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>What even is all this? Looks like some really retro footage...</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Peris's reaction to the glitch. She does not register the spiral as an intrusion at all; she takes it for part of the footage, just more dated, odd wellness video. The dark irony is that the capture motif surfaces right in front of her and reads to her as nothing, content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>peris_sim.worker.okay</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>WORKER</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Hey, we detected abnormal vital signals. Let's get you looked at.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Adjacent worker reacts as Peris removes the sim equipment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>peris_sim.worker.medical</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>WORKER</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>Yikes, got sanctioned? How boring. The med bay's a snoozefest. I don't remember a thing!</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>The workplace reads refusal as a medical problem.</t>
         </is>

</xml_diff>

<commit_message>
checkpoint Godot 4.7 gameplay and authored-scene work
Checkpoint the accumulated migration, generation, level, playthrough, shader, model-import, and authored UI work. Ignore local QA capture output while preserving its files on disk. Focused authored-UI/elevator/builder suites pass 450/450; the full branch suite currently reports 16458 passes and 39 known cross-system failures, so this is intentionally a preservation checkpoint rather than a release-green claim.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
+++ b/to-rust-as-we-fall/data/dialogue/en/act1.xlsx
@@ -12491,12 +12491,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>The corridor opens onto a walkway, an open span over a deeper dark. Half the railing is gone. Down in the gloom below, shapes that were people.</t>
+          <t>The corridor opens onto an intact walkway, an open span over a deeper dark. At the far end, a Chembrane seal blocks the way. Down in the gloom below, shapes that were people.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Bridge description. The fork branches off below this walkway; the party passes directly above it here and sees the enemies and the bodies in the gloom below. The far end of the span gives way and drops them to that sub-level fork. (see GDD 9.5)</t>
+          <t>Bridge description. The fork branches off below this walkway; the party passes directly above it here and sees the enemies and the bodies in the gloom below. The intact span reaches a blocked Chembrane seal; the deck gives way around two-thirds across and drops them to that sub-level fork. (see GDD 9.5)</t>
         </is>
       </c>
     </row>
@@ -12523,7 +12523,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>...Oh my god, Aster, are these people? That lump's got a broken device, and there's bits of Wonderweave strewn about...</t>
+          <t>...Oh my god, Aster, are these people? That lump's got a broken device, and there's bits of Chembrane strewn about...</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">

</xml_diff>